<commit_message>
Stage 8 review fixes: E-005
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/IS3/WA-2018-082/Results/Approved/IS3_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Stability/IS3/WA-2018-082/Results/Approved/IS3_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -173,7 +173,7 @@
   <commentList>
     <comment ref="A6" authorId="0" shapeId="0">
       <text>
-        <t>Istravune QA to be sent the signed copy with the shelf-life justification.</t>
+        <t>Send the signed report with the shelf-life justification.</t>
       </text>
     </comment>
   </commentList>
@@ -610,7 +610,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Twenty-four-month ICH stability of IS-3 tablets, with the HPLC assay and related-substances method qualified before the first pull. Pulls to 24 months; interim review completed 30 Apr 2019.</t>
+          <t>Twenty-four-month ICH stability of IS-3 tablets, with assay and related-substances qualification. Pulls to 24 months; interim review completed 30 Apr 2019.</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Assay as % label claim (HPLC). Impurities as % area. Water by Karl Fischer. Pulls from the ICH chamber programme as recorded on the batch card.</t>
+          <t>Assay as % label claim (HPLC). Impurities as % area. Water by Karl Fischer. Pulls from the ICH chamber programme as recorded on the batch card. Time zero is one initial analysis shared by all storage conditions; repeated initial rows do not represent separate pulls.</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Validated before the first stability pull under the assay and related-substances validation protocol. Acceptance criteria as written in the protocol.</t>
+          <t>Assay and related-substances validation parameters and their acceptance criteria are summarised below.</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1583,14 +1583,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Long-term data at 25 °C/60% RH support the proposed shelf life to the final pull. Accelerated data follow the same trend and do not change the conclusion.</t>
+          <t>Long-term data at 25 °C/60% RH support the proposed shelf life within the tested interval. Intermediate data also extend to the final reported timepoint; accelerated results stop at six months and show greater impurity growth. All reported pulls comply.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>The final pull was assayed against the same system suitability criteria as the first pull. The method was not changed over the programme.</t>
+          <t>The method validation parameters meet their stated acceptance criteria. The project review concluded that the method remained suitable through the final pull; sequence-specific checks remain in the approved sequence sheets.</t>
         </is>
       </c>
     </row>
@@ -1598,34 +1598,24 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>Review responsibility</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>By</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
+          <t>Person</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Data review</t>
+          <t>Stability review</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Dr L. Wu</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>30 Apr 2020</t>
         </is>
       </c>
     </row>
@@ -1640,26 +1630,16 @@
           <t>S. Mahmood</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>30 Apr 2020</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Approval</t>
+          <t>Protocol lead</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Dr A. Penrose</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>30 Apr 2020</t>
         </is>
       </c>
     </row>

</xml_diff>